<commit_message>
update capitulo precio leche
</commit_message>
<xml_diff>
--- a/datos/2026-02-01-precio-leche.xlsx
+++ b/datos/2026-02-01-precio-leche.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/34bf2af71bbc2e43/Documentos/GitHub/master-queseria/website/datos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="8_{C3D8DB6E-80F1-4A74-A94C-632DB8A5E2B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2973D2D8-44DD-45D7-9D0B-35010ABC7397}"/>
+  <xr:revisionPtr revIDLastSave="35" documentId="8_{C3D8DB6E-80F1-4A74-A94C-632DB8A5E2B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{275DC052-7D4B-4071-AB00-637E9DC17868}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="675" activeTab="1" xr2:uid="{6977E7F1-D64B-47FE-B2A7-D4E9B0399E18}"/>
   </bookViews>
@@ -725,11 +725,11 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="6">
     <numFmt numFmtId="164" formatCode="#,##0_ ;[Red]\-#,##0\ "/>
-    <numFmt numFmtId="167" formatCode="0.000"/>
-    <numFmt numFmtId="168" formatCode="_-* #,##0.00\ _€_-;\-* #,##0.00\ _€_-;_-* &quot;-&quot;??\ _€_-;_-@_-"/>
-    <numFmt numFmtId="169" formatCode="#,##0.00_ ;[Red]\-#,##0.00\ "/>
-    <numFmt numFmtId="171" formatCode="0.0000"/>
-    <numFmt numFmtId="172" formatCode="0.0000_ ;[Red]\-0.0000\ "/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="_-* #,##0.00\ _€_-;\-* #,##0.00\ _€_-;_-* &quot;-&quot;??\ _€_-;_-@_-"/>
+    <numFmt numFmtId="167" formatCode="#,##0.00_ ;[Red]\-#,##0.00\ "/>
+    <numFmt numFmtId="168" formatCode="0.0000"/>
+    <numFmt numFmtId="169" formatCode="0.0000_ ;[Red]\-0.0000\ "/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
@@ -952,11 +952,11 @@
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -973,7 +973,7 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
@@ -997,16 +997,16 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1031,12 +1031,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
@@ -1045,16 +1045,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1069,19 +1069,19 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="171" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="169" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="169" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1090,14 +1090,15 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="172" fontId="0" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="0" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="2" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="2" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="2" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="2" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="2" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="172" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Millares 2" xfId="2" xr:uid="{0DF497A4-B1A4-4A8E-B2C1-3A725AAFDCC2}"/>
@@ -3823,7 +3824,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5C6A5F7-7476-41E2-B25E-833B29F6911A}">
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="40.28515625" customWidth="1"/>
@@ -4150,23 +4151,27 @@
       <c r="D30" s="10"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B31" s="10"/>
-      <c r="C31" s="10"/>
       <c r="D31" s="10"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B32" s="10"/>
-      <c r="C32" s="10"/>
       <c r="D32" s="10"/>
     </row>
-    <row r="33" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D33" s="10"/>
     </row>
-    <row r="34" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B34" s="63"/>
       <c r="D34" s="10"/>
     </row>
-    <row r="35" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B35" s="10"/>
       <c r="D35" s="10"/>
+    </row>
+    <row r="36" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B36" s="10"/>
+    </row>
+    <row r="37" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B37" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>